<commit_message>
config: 扩充 EnemyEntityTable 增加3个敌人预设
新增普通-容易(ID2)、普通-普通(ID3)、精英-困难(ID4)三种敌人配置。
调整ID1后羿测试敌人的警觉参数（AlertDistance/AlertTime/DetectDistance/CombatDistance）。
</commit_message>
<xml_diff>
--- a/AAAGameData/DataTables/EnemyEntityTable.xlsx
+++ b/AAAGameData/DataTables/EnemyEntityTable.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="73">
   <si>
     <t>#</t>
   </si>
@@ -228,6 +228,24 @@
   </si>
   <si>
     <t>测试</t>
+  </si>
+  <si>
+    <t>普通敌人-容易</t>
+  </si>
+  <si>
+    <t>容易难度</t>
+  </si>
+  <si>
+    <t>普通敌人-普通</t>
+  </si>
+  <si>
+    <t>普通难度</t>
+  </si>
+  <si>
+    <t>精英敌人-困难</t>
+  </si>
+  <si>
+    <t>困难难度</t>
   </si>
 </sst>
 </file>
@@ -240,7 +258,14 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -696,148 +721,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1192,13 +1217,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AE5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="4"/>
+  <dimension ref="A1:AE8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="7"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="8" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
     <col min="5" max="5" width="8" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
     <col min="7" max="7" width="11" customWidth="1"/>
@@ -1593,7 +1618,7 @@
         <v>10</v>
       </c>
       <c r="R5" s="1">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="S5" s="1">
         <v>1.5</v>
@@ -1614,13 +1639,13 @@
         <v>1</v>
       </c>
       <c r="Y5" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="Z5" s="1">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="AA5" s="1">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="AB5" s="1">
         <v>4</v>
@@ -1629,10 +1654,283 @@
         <v>20</v>
       </c>
       <c r="AD5" s="1">
+        <v>3</v>
+      </c>
+      <c r="AE5" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" spans="1:31">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1">
         <v>2</v>
       </c>
-      <c r="AE5" s="1">
-        <v>1</v>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E6" s="1">
+        <v>11001</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G6" s="1">
+        <v>0</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0</v>
+      </c>
+      <c r="I6" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J6" s="1">
+        <v>0</v>
+      </c>
+      <c r="K6" s="1">
+        <v>1</v>
+      </c>
+      <c r="L6" s="1">
+        <v>2601</v>
+      </c>
+      <c r="M6" s="1">
+        <v>1</v>
+      </c>
+      <c r="N6" s="1">
+        <v>8</v>
+      </c>
+      <c r="O6" s="1">
+        <v>1.8</v>
+      </c>
+      <c r="P6" s="1">
+        <v>0.4</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>8</v>
+      </c>
+      <c r="R6" s="1">
+        <v>20</v>
+      </c>
+      <c r="S6" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="T6" s="1">
+        <v>60</v>
+      </c>
+      <c r="U6" s="1">
+        <v>8</v>
+      </c>
+      <c r="V6" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="W6" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="X6" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y6" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="Z6" s="1">
+        <v>10</v>
+      </c>
+      <c r="AA6" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="AB6" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="AC6" s="1">
+        <v>25</v>
+      </c>
+      <c r="AD6" s="1">
+        <v>4</v>
+      </c>
+      <c r="AE6" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1" spans="1:31">
+      <c r="A7" s="1"/>
+      <c r="B7" s="1">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E7" s="1">
+        <v>11001</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0</v>
+      </c>
+      <c r="I7" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J7" s="1">
+        <v>0</v>
+      </c>
+      <c r="K7" s="1">
+        <v>1</v>
+      </c>
+      <c r="L7" s="1">
+        <v>2601</v>
+      </c>
+      <c r="M7" s="1">
+        <v>1</v>
+      </c>
+      <c r="N7" s="1">
+        <v>10</v>
+      </c>
+      <c r="O7" s="1">
+        <v>2</v>
+      </c>
+      <c r="P7" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="Q7" s="1">
+        <v>10</v>
+      </c>
+      <c r="R7" s="1">
+        <v>15</v>
+      </c>
+      <c r="S7" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="T7" s="1">
+        <v>60</v>
+      </c>
+      <c r="U7" s="1">
+        <v>8</v>
+      </c>
+      <c r="V7" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="W7" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="X7" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y7" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="1">
+        <v>8</v>
+      </c>
+      <c r="AA7" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="AB7" s="1">
+        <v>4</v>
+      </c>
+      <c r="AC7" s="1">
+        <v>20</v>
+      </c>
+      <c r="AD7" s="1">
+        <v>3</v>
+      </c>
+      <c r="AE7" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" spans="1:31">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1">
+        <v>4</v>
+      </c>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E8" s="1">
+        <v>11001</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1</v>
+      </c>
+      <c r="H8" s="1">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" s="1">
+        <v>18</v>
+      </c>
+      <c r="K8" s="1">
+        <v>2</v>
+      </c>
+      <c r="L8" s="1">
+        <v>2601</v>
+      </c>
+      <c r="M8" s="1">
+        <v>1</v>
+      </c>
+      <c r="N8" s="1">
+        <v>12</v>
+      </c>
+      <c r="O8" s="1">
+        <v>2.5</v>
+      </c>
+      <c r="P8" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="Q8" s="1">
+        <v>12</v>
+      </c>
+      <c r="R8" s="1">
+        <v>12</v>
+      </c>
+      <c r="S8" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="T8" s="1">
+        <v>60</v>
+      </c>
+      <c r="U8" s="1">
+        <v>8</v>
+      </c>
+      <c r="V8" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="W8" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="X8" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y8" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="Z8" s="1">
+        <v>5</v>
+      </c>
+      <c r="AA8" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="AB8" s="1">
+        <v>5</v>
+      </c>
+      <c r="AC8" s="1">
+        <v>18</v>
+      </c>
+      <c r="AD8" s="1">
+        <v>2</v>
+      </c>
+      <c r="AE8" s="1">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>